<commit_message>
Update setup-sheet.gs — 26 cols matching API
</commit_message>
<xml_diff>
--- a/WE_Schools_v2.xlsx
+++ b/WE_Schools_v2.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="57">
   <si>
     <t>رقم الطلب</t>
   </si>
@@ -104,55 +104,37 @@
     <t>القيمة</t>
   </si>
   <si>
-    <t>إجمالي المتقدمين</t>
-  </si>
-  <si>
-    <t>=COUNTA(Applications!A2:A1048576)</t>
-  </si>
-  <si>
-    <t>عدد المقبولين</t>
-  </si>
-  <si>
-    <t>=COUNTIF(K2:K1048576,"قيد المراجعة")</t>
-  </si>
-  <si>
-    <t>عدد المرفوضين</t>
-  </si>
-  <si>
-    <t>=COUNTIF(K2:K1048576,"مقبول")</t>
-  </si>
-  <si>
-    <t>قيد المراجعة</t>
-  </si>
-  <si>
-    <t>=COUNTIF(K2:K1048576,"مرفوض")</t>
-  </si>
-  <si>
-    <t>ناقص مستندات</t>
-  </si>
-  <si>
-    <t>=COUNTIF(K2:K1048576,"ناقص مستندات")</t>
-  </si>
-  <si>
-    <t>بانتظار التواصل</t>
-  </si>
-  <si>
-    <t>=COUNTIF(K2:K1048576,"بانتظار التواصل")</t>
-  </si>
-  <si>
-    <t>الطلاب حسب المحافظة</t>
+    <t>📋 إجمالي المتقدمين</t>
+  </si>
+  <si>
+    <t>🟢 عدد المقبولين</t>
+  </si>
+  <si>
+    <t>🔴 عدد المرفوضين</t>
+  </si>
+  <si>
+    <t>🟡 قيد المراجعة</t>
+  </si>
+  <si>
+    <t>🟠 ناقص مستندات</t>
+  </si>
+  <si>
+    <t>⏳ بانتظار التواصل</t>
+  </si>
+  <si>
+    <t>🏫 توزيع المدارس</t>
+  </si>
+  <si>
+    <t>المدرسة</t>
   </si>
   <si>
     <t>العدد</t>
   </si>
   <si>
-    <t>الطلاب حسب المدرسة</t>
-  </si>
-  <si>
-    <t>المدرسة</t>
-  </si>
-  <si>
-    <t>🔍 اكتب رقم الطلب</t>
+    <t>🌍 توزيع المحافظات</t>
+  </si>
+  <si>
+    <t>🔍 اكتب رقم الطلب في الخلية B2</t>
   </si>
   <si>
     <t>شهادة الميلاد</t>
@@ -170,46 +152,37 @@
     <t>ملف التقديم</t>
   </si>
   <si>
-    <t>المؤشر</t>
+    <t>📊 بطاقات الأداء</t>
+  </si>
+  <si>
+    <t>📈 مؤشرات الأداء</t>
+  </si>
+  <si>
+    <t>📅 التسجيلات اليومية</t>
+  </si>
+  <si>
+    <t>📋 إجمالي الطلبات</t>
+  </si>
+  <si>
+    <t>آخر تسجيل</t>
   </si>
   <si>
     <t>التاريخ</t>
   </si>
   <si>
-    <t>عدد المتقدمين</t>
-  </si>
-  <si>
-    <t>📋 إجمالي الطلبات</t>
-  </si>
-  <si>
-    <t>📊 مؤشرات الأداء</t>
-  </si>
-  <si>
-    <t>📈 بيانات الرسم البياني</t>
-  </si>
-  <si>
     <t>🟢 المقبولين</t>
   </si>
   <si>
-    <t>آخر تسجيل</t>
-  </si>
-  <si>
-    <t>استخدم PivotTable للرسوم البيانية</t>
+    <t>أول تسجيل</t>
   </si>
   <si>
     <t>🔴 المرفوضين</t>
   </si>
   <si>
-    <t>أول تسجيل</t>
+    <t>متوسط التسجيل يوميًا</t>
   </si>
   <si>
     <t>🟡 تحت المراجعة</t>
-  </si>
-  <si>
-    <t>متوسط التسجيل يوميًا</t>
-  </si>
-  <si>
-    <t>🟠 ناقص مستندات</t>
   </si>
   <si>
     <t>نسبة اكتمال البيانات</t>
@@ -236,32 +209,37 @@
     <font>
       <b/>
       <color rgb="1E3A5F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="1E3A5F"/>
       <sz val="16"/>
     </font>
     <font>
       <b/>
       <color rgb="1E7E1E"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
       <color rgb="B82424"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
       <color rgb="AB7F12"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
       <color rgb="CC6600"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
       <color rgb="6B7280"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
@@ -274,12 +252,17 @@
     <font>
       <b/>
       <color rgb="1E3A5F"/>
-      <sz val="12"/>
+      <sz val="18"/>
     </font>
     <font>
       <b/>
       <color rgb="1E3A5F"/>
-      <sz val="18"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0D9488"/>
+      <sz val="13"/>
     </font>
     <font>
       <b/>
@@ -290,16 +273,6 @@
       <b/>
       <color rgb="1E7E1E"/>
       <sz val="18"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="0D9488"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="6B7280"/>
-      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -402,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -413,38 +386,46 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1204,11 +1185,11 @@
   <sheetPr>
     <tabColor rgb="C8952E"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1220,90 +1201,96 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4">
+        <f>=COUNTA(Applications!A2:A1048576)</f>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="6">
+        <f>=COUNTIF(K2:K1048576,"مقبول")</f>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="7">
+        <f>=COUNTIF(K2:K1048576,"مرفوض")</f>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B5" s="8">
+        <f>=COUNTIF(K2:K1048576,"قيد المراجعة")</f>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B6" s="9">
+        <f>=COUNTIF(K2:K1048576,"ناقص مستندات")</f>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="B7" s="10">
+        <f>=COUNTIF(K2:K1048576,"بانتظار التواصل")</f>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="7" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B10" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="8" t="s">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="12">
+        <f>IFERROR(INDEX(Applications!$D$2:$D$9999, MATCH(0, INDEX(COUNTIF($A$10:$A10, Applications!$D$2:$D$9999), 0), 0)), "")</f>
+      </c>
+      <c r="B11" s="12">
+        <f>IF(A11="","",COUNTIF(Applications!$D$2:$D$9999, A11))</f>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D8" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9">
-        <f>IFERROR(INDEX(Applications!$F$2:$F$9999, MATCH(0, COUNTIF($D$8:$D8, Applications!$F$2:$F$9999), 0)), "")</f>
-      </c>
-      <c r="E9">
-        <f>IF(D9="","",COUNTIF(Applications!$F$2:$F$9999, D9))</f>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
-        <f>IFERROR(INDEX(Applications!$D$2:$D$9999, MATCH(0, COUNTIF($A$10:$A10, Applications!$D$2:$D$9999), 0)), "")</f>
-      </c>
-      <c r="B11" s="4">
-        <f>IF(A11="","",COUNTIF(Applications!$D$2:$D$9999, A11))</f>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="12">
+        <f>IFERROR(INDEX(Applications!$F$2:$F$9999, MATCH(0, INDEX(COUNTIF($A$14:$A14, Applications!$F$2:$F$9999), 0), 0)), "")</f>
+      </c>
+      <c r="B15" s="12">
+        <f>IF(A15="","",COUNTIF(Applications!$F$2:$F$9999, A15))</f>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1421,16 +1408,16 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f>IFERROR(VLOOKUP($B$2, Applications!$A$2:$Z$9999, COLUMN(A1), FALSE), "")</f>
+        <f>IFERROR(VLOOKUP($B$2, Applications!$A$2:$Z$9999, 1, FALSE), "")</f>
       </c>
       <c r="B3">
         <f>IFERROR(VLOOKUP($B$2, Applications!$A$2:$Z$9999, 2, FALSE), "")</f>
@@ -1536,19 +1523,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1603,28 +1590,27 @@
   <sheetPr>
     <tabColor rgb="8B5CF6"/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="3" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="3" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="3" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="4" customWidth="1"/>
+    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="4" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="3" customWidth="1"/>
+    <col min="12" max="12" width="4" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>28</v>
@@ -1633,7 +1619,7 @@
         <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>28</v>
@@ -1642,145 +1628,142 @@
         <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="16">
+        <f>=Statistics!B2</f>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="18">
+        <f>=MAX(Applications!L2:L1048576)</f>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="N2" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="21">
+        <f>=Statistics!B3</f>
+      </c>
+      <c r="D3" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="E3" s="18">
+        <f>=MIN(Applications!L2:L1048576)</f>
+      </c>
+      <c r="G3">
+        <f>IFERROR(INDEX(Applications!$L$2:$L$9999, MATCH(0, INDEX(COUNTIF($G$2:$G2, Applications!$L$2:$L$9999), 0), 0)), "")</f>
+      </c>
+      <c r="H3">
+        <f>IF(G3="","",COUNTIF(Applications!$L$2:$L$9999, G3))</f>
+      </c>
+      <c r="J3">
+        <f>=Statistics!A11:A1048576</f>
+      </c>
+      <c r="K3">
+        <f>=Statistics!B11:B1048576</f>
+      </c>
+      <c r="M3">
+        <f>=Statistics!A15:A1048576</f>
+      </c>
+      <c r="N3">
+        <f>=Statistics!B15:B1048576</f>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="B4" s="23">
+        <f>=Statistics!B4</f>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="14">
-        <f>=Statistics!B2</f>
-      </c>
-      <c r="D2" s="13" t="s">
+      <c r="E4" s="18">
+        <f>=IFERROR(ROUND(Statistics!B2/MAX(DAYS(MAX(Applications!L2:L1048576),MIN(Applications!L2:L1048576)),1),1),0)</f>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="J2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="M2" s="15" t="s">
+      <c r="B5" s="25">
+        <f>=Statistics!B5</f>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="17">
-        <f>=Statistics!B3</f>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="18">
-        <f>=MAX(Applications!L2:L1048576)</f>
-      </c>
-      <c r="G3">
-        <f>=Statistics!A11:A</f>
-      </c>
-      <c r="H3">
-        <f>=Statistics!B11:B</f>
-      </c>
-      <c r="J3">
-        <f>=Statistics!D9:D</f>
-      </c>
-      <c r="K3">
-        <f>=Statistics!E9:E</f>
-      </c>
-      <c r="M3" s="19" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="21">
-        <f>=Statistics!B4</f>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="18">
-        <f>=MIN(Applications!L2:L1048576)</f>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="23">
-        <f>=Statistics!B5</f>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>63</v>
-      </c>
       <c r="E5" s="18">
-        <f>=IFERROR(ROUND(Statistics!B2/MAX(DAYS(MAX(Applications!L2:L1048576),MIN(Applications!L2:L1048576)),1),1),0)</f>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="25">
+        <f>=IFERROR(ROUND(COUNTIF(Applications!A2:A1048576,"&lt;&gt;")/COUNTA(Applications!A2:A1048576)*100,1)&amp;"%","0%")</f>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="27">
         <f>=Statistics!B6</f>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="18">
-        <f>=IFERROR(ROUND(COUNTIF(Applications!A2:A1048576,"&lt;&gt;")/COUNTA(Applications!A2:A1048576)*100,1)&amp;"%","0%")</f>
-      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="27">
+      <c r="A7" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="29">
         <f>=Statistics!B7</f>
       </c>
     </row>
-    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>